<commit_message>
Atualização de documentação e outras mudanças
</commit_message>
<xml_diff>
--- a/backend/benchmark/results/arquivos_gerados_benchmark/gastos.xlsx
+++ b/backend/benchmark/results/arquivos_gerados_benchmark/gastos.xlsx
@@ -417,12 +417,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -436,11 +435,6 @@
           <t>Valor</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Categoria</t>
-        </is>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>